<commit_message>
Leads: 2026-09-29 00:20 UTC (cycle 3)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://jandjheatingandairconditioning.com/air-conditioning-repair-athens-ga/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>jandjacdoctor@aol.com</t>
@@ -614,6 +613,62 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Rocky Top Total Roofing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>rockytoptotalroofing.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://rockytoptotalroofing.com/services</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>sales@rockytoptotalroofing.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>(970) 658-5881</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>residential roofing company Fort Collins CO</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 00:24 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -639,7 +639,6 @@
           <t>https://rockytoptotalroofing.com/services</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>sales@rockytoptotalroofing.com</t>
@@ -669,6 +668,62 @@
         </is>
       </c>
       <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Road Roofing + Construction LLC</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>roadroofing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://www.roadroofing.com/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>service@roadroofing.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(972) 217-2690</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Garland TX</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>90</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>residential roofing company Garland TX</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 00:26 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -694,7 +694,6 @@
           <t>https://www.roadroofing.com/</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>service@roadroofing.com</t>
@@ -724,6 +723,66 @@
         </is>
       </c>
       <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Plumbing Sarasota</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>plumbingsarasotaflorida.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://plumbingsarasotaflorida.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Service Award</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>info@plumbingsarasota.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(941) 477-1334</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>plumber Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 00:32 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -788,6 +788,62 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>YourHVACGuy</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>hireyourhvacguy.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://www.hireyourhvacguy.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>support@hireyourhvacguy.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>815.276.3166</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Aurora IL</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>98</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>HVAC contractor Aurora IL</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 00:33 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -809,7 +809,6 @@
           <t>https://www.hireyourhvacguy.com/</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>support@hireyourhvacguy.com</t>
@@ -839,6 +838,66 @@
         </is>
       </c>
       <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Cornerstone Roofing &amp; Restoration</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>csrr-colorado.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://csrr-colorado.com/service-areas/aurora-co</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Colorado Springs</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>admin@csrr-co.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>(719) 600-7852</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>90</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>residential roofing company Aurora CO</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 00:35 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -903,6 +903,66 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Roofing Contractors in Washington, DC | United Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>unitedroofingdc.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://www.unitedroofingdc.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Why Washington</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>unitedroofingdc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(202) 710-9160</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Washington DC</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>86</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>roofing contractor Washington DC</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 00:59 UTC (cycle 30)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -963,6 +963,66 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Metal Roofing in Long Beach</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>milianroofing.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://milianroofing.com/locations/long-beach-ca/metal-roofing</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Material Warranties</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@milianroofing.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(213) 758-0798</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Long Beach CA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>90</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Long Beach CA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:10 UTC (cycle 37)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1023,6 +1023,66 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AC Repair Grand Rapids MI | Same-Day AC Repair in Grand Rapids &amp; West Michigan</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>acrepairgrandrapids.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://acrepairgrandrapids.com/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Repair Grand</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ops@acrepairgrandrapids.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(888) 217-1674</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>90</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>air conditioning repair Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:13 UTC (cycle 39)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1083,6 +1083,126 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Carrier Ductless | Clean Electric Heat Pumps</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ductlesscarrier.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://ductlesscarrier.com/lancaster-pa/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Inflation Reduction</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>dcl@peirce.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(267) 668-3474</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Lancaster PA</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>heat pump installation Lancaster PA</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Summers &amp; Zim\'s</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>sumzim.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://sumzim.com/services/heating/heat-pump-repair-and-replacement/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Team Talk</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@sumzim.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>610-593-5129</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Lancaster PA</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>90</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>heat pump installation Lancaster PA</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:16 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1203,6 +1203,66 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Altair Roofing The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>roofingthewoodlandstx.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://roofingthewoodlandstx.com/services/roof-repair-the-woodlands-tx</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Altair Roofing</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>support@roofingthewoodlandstx.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(346) 540-4717</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>roof repair company The Woodlands TX</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:28 UTC (cycle 49)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1263,6 +1263,66 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Inside Out Plumbing, LLC</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>insideoutplumbers.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://www.insideoutplumbers.com/norfolk-va/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Chesapeake Bay</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>john@smith.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(757) 882-0728</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Norfolk VA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>plumbing company Norfolk VA</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:31 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1323,6 +1323,66 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>St. Charles MO Roofing Contractor | SuperRoofer Exteriors LLC</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>superrooferstl.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>https://superrooferstl.com/locations/st-charles-mo</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Team Darien</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>asuperroofer@gmail.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>314-422-4704</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>St Charles MO</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>90</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>roofer St Charles MO</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:32 UTC (cycle 52)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1383,6 +1383,126 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Emergency Plumbers NJ</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>emergencyplumbersnj.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://emergencyplumbersnj.com/passaic-county/emergency-plumber-paterson-nj/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Why Homeowners</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>cityservicegroupnj@gmail.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>973-604-3856</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Paterson NJ</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>emergency plumber Paterson NJ</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>BUILT Roofing</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>builtroofingaz.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://builtroofingaz.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Starts With</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>jakep@builtroofingaz.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>480-650-9005</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>98</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>roofer Gilbert AZ</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:38 UTC (cycle 56)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1503,6 +1503,66 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Frisco Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>friscoheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://friscoheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Frisco Heating</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>contact@friscoheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>972-954-4543</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>heating and cooling company Frisco TX</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:40 UTC (cycle 57)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1563,6 +1563,66 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Kyzar Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>kyzarairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://kyzarairconditioning.com/service-areas/ac-repair-hollywood-fl/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Top Rated</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>service@kyzarairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>(561) 640-1000</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Hollywood FL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>air conditioning repair Hollywood FL</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:44 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1623,6 +1623,66 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Metal Roof Installation | Elgin &amp; Chicagoland</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>lakeshorebuildersrestoration.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.lakeshorebuildersrestoration.com/metal-roof-installation</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>info@lakeshorebuildersrestoration.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(847) 348-9868</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Elgin IL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Elgin IL</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 01:56 UTC (cycle 68)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1683,6 +1683,66 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>BEENE Plumbing Contractor</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>beene.cc</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://beene.cc/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Broken Arrow</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>service@beene.cc</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>918-451-9081</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>100</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>plumbing company Broken Arrow OK</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:03 UTC (cycle 73)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1743,6 +1743,126 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>About Sewer</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>clarksvilletn.gov</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://www.clarksvilletn.gov/307/About-Sewer</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Mark Riggins</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>gasandwater@cityofclarksville.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(931) 553-2424</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Clarksville TN</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>100</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>sewer repair Clarksville TN</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Accu Air - No #1 HVAC Company in Tulsa</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>accuairok.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>https://accuairok.com/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Top Rated</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>info@accuairok.com</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>(918) 321-7933</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Tulsa OK</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>98</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>AC installation Tulsa OK</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:06 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1863,6 +1863,66 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Ac And Heat Replacement Greenville, SC | Phoenix HVAC</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>phoenixairsc.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>https://www.phoenixairsc.com/contact/ac-and-heat-replacement-greenville</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Signs It</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>derekmcalhany@gmail.com</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>(864) 318-6276</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>100</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>AC installation Greenville SC</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:09 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1923,6 +1923,58 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Roofer | McDermaid Roofing &amp; Insulating Co | Rockford, IL</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>mcdermaidroofing.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>https://www.mcdermaidroofing.com/</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>mcroof@mcdermaidroofing.com</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Rockford IL</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>72</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>roofer Rockford IL</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:16 UTC (cycle 82)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1944,13 +1944,11 @@
           <t>https://www.mcdermaidroofing.com/</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>mcroof@mcdermaidroofing.com</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>Rockford IL</t>
@@ -1970,6 +1968,62 @@
         </is>
       </c>
       <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Reliable Comfort</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>reliablecomfort.com</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>https://www.reliablecomfort.com/service-area/bloomington-in/</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>info@reliablecomfort.com</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>(812) 372-8011</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Bloomington IN</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>100</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>heating and cooling company Bloomington IN</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:37 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L27"/>
+  <dimension ref="A1:L28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1994,7 +1994,6 @@
           <t>https://www.reliablecomfort.com/service-area/bloomington-in/</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>info@reliablecomfort.com</t>
@@ -2024,6 +2023,62 @@
         </is>
       </c>
       <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>New AC &amp; Heating Installations | Stockton, CA | Guerrero's</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>guerrerosheatingandair.net</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>https://www.guerrerosheatingandair.net/air-conditioners-heating-installation</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>guerreroshvac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(209) 482-1818</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Stockton CA</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>90</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>heat pump installation Stockton CA</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:38 UTC (cycle 97)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2049,7 +2049,6 @@
           <t>https://www.guerrerosheatingandair.net/air-conditioners-heating-installation</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>guerreroshvac@gmail.com</t>
@@ -2079,6 +2078,126 @@
         </is>
       </c>
       <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>https://pasadenaroofingpro.com/</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>pasadenaroofingpro.com</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>https://www.pasadenaroofingpro.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Commercial Roofing</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>admin@pasadenaroofingpro.com</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>626-669-1637</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>100</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Metal Roofing Installation in Pasadena, TX | Tell Project Roofing</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>roofing.tellprojectstx.com</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>https://roofing.tellprojectstx.com/metal-roofing-pasadena.html</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Full Texas</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>info@tellprojectstx.com</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>(832) 591-7991</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Pasadena TX</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>90</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Pasadena TX</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:41 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L30"/>
+  <dimension ref="A1:L32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2203,6 +2203,122 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Big Will's AC and Heating</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>bigwillsacandheating.com</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>https://www.bigwillsacandheating.com/hvac-services/heat-pump-service/</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Big Will</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>willanglinais@gmail.com</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>(337) 962-8632</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Lafayette LA</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>90</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>heat pump installation Lafayette LA</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Metal Roofing Installation in Duluth, MN</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>forevernorthroofing.com</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>https://www.forevernorthroofing.com/service-area/duluth-mn</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>joe@forevernorthroofing.com</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>(218) 409-0246</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>90</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Duluth MN</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:46 UTC (cycle 102)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L32"/>
+  <dimension ref="A1:L33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2284,7 +2284,6 @@
           <t>https://www.forevernorthroofing.com/service-area/duluth-mn</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>joe@forevernorthroofing.com</t>
@@ -2314,6 +2313,66 @@
         </is>
       </c>
       <c r="L32" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Our Place Air &amp; Home Repair</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>callourplace.com</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>https://callourplace.com/drain-cleaning-orlando/</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Reviews Thousands</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>info@callourplace.com</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>800-291-0949</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>90</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>drain cleaning service Orlando FL</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:47 UTC (cycle 103)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2378,6 +2378,62 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Water Heater Repair - Boulder, CO - Bernie's Plumbing</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>berniesplumbing.com</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>https://www.berniesplumbing.com/water-heater-solutions-boulder</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>info@berniesplumbing.com</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>(303) 442-7060</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Boulder CO</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>88</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>water heater repair Boulder CO</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:55 UTC (cycle 108)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L34"/>
+  <dimension ref="A1:L35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2399,7 +2399,6 @@
           <t>https://www.berniesplumbing.com/water-heater-solutions-boulder</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>info@berniesplumbing.com</t>
@@ -2429,6 +2428,66 @@
         </is>
       </c>
       <c r="L34" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Win Mechanical</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>winmechanical.com</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>https://www.winmechanical.com/service-areas/lewiston</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Efficiency Maine</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>info@winmechanical.com</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>(207) 481-3675</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Lewiston ME</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>90</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lewiston ME</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:56 UTC (cycle 109)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L35"/>
+  <dimension ref="A1:L36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2493,6 +2493,62 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Plumbing Service &amp; Repair - Woodbridge, New Jersey - Owen S. Dunigan &amp; Co., Inc.</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>duniganplumbingnj.com</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>https://www.duniganplumbingnj.com/</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>duniganplumbing@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>732-634-0630</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
+        <v>90</v>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>plumbing company Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 02:59 UTC (cycle 111)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L36"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2514,7 +2514,6 @@
           <t>https://www.duniganplumbingnj.com/</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>duniganplumbing@yahoo.com</t>
@@ -2544,6 +2543,66 @@
         </is>
       </c>
       <c r="L36" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair in Fort Lauderdale, FL | Moody Plumbing</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>moodyplumbing.com</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>https://www.moodyplumbing.com/sewer-line-repair-fort-lauderdale-fl</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>admin@moodyplumbing.com</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>954-972-1079</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
+        <v>84</v>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>sewer repair Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 03:33 UTC (cycle 134)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L37"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2608,6 +2608,182 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>In &amp; Out Plumbing</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>inandoutplumbingcny.com</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>https://inandoutplumbingcny.com/</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>inandoutplumbingcny@gmail.com</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>315-489-4486</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Syracuse NY</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>100</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>plumbing company Syracuse NY</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Titanium Roofing Experts</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>titaniumroofingexperts.com</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>https://titaniumroofingexperts.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Commercial Licensed</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>info@titaniumroofingexperts.com</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>(941) 216-5705</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>100</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LONGBOAT KEY ROOFING</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>longboatkeyroofing.net</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>https://www.longboatkeyroofing.net/metal-roofing-contractors/</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Longboat Key</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>admin@longboatkeyroofing.net</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>941-706-4170</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Sarasota FL</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>90</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Sarasota FL</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 03:37 UTC (cycle 137)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L40"/>
+  <dimension ref="A1:L41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2629,7 +2629,6 @@
           <t>https://inandoutplumbingcny.com/</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>inandoutplumbingcny@gmail.com</t>
@@ -2779,6 +2778,66 @@
         </is>
       </c>
       <c r="L40" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Amped Home Services</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ampedhomeservices.com</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>https://ampedhomeservices.com/norman-oklahoma-sewer-drain-repair/</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Oklahoma Built</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>contact@ampedhomeservices.com</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>(405) 506-9082</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Norman OK</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>96</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>sewer repair Norman OK</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 03:40 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2843,6 +2843,122 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Sewer Line Repair in Sterling Heights</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>austinsmithplumbing.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>https://www.austinsmithplumbing.com/locations/sterling-heights-mi/sewer-line-repair</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>info@austinsmithplumbing.com</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>(877) 697-1160</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>90</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>sewer repair Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Roof Replacement in Charlotte, NC</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>persevereroofing.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>https://www.persevereroofing.com/roof-replacement</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Avg Rating</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>info@persevereroofing.com</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>(704) 498-2930</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Charlotte NC</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>90</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>roof replacement Charlotte NC</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 03:46 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2864,7 +2864,6 @@
           <t>https://www.austinsmithplumbing.com/locations/sterling-heights-mi/sewer-line-repair</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>info@austinsmithplumbing.com</t>
@@ -2954,6 +2953,66 @@
         </is>
       </c>
       <c r="L43" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Dura Pier Foundation Repair</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>durapier.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>https://durapier.com/dallas/sewer-line-repair/</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Expert Under</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>info@durapier.com</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>(214) 699-4784</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>94</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>sewer repair Dallas TX</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 03:48 UTC (cycle 144)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L44"/>
+  <dimension ref="A1:L45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3018,6 +3018,66 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Haven Studios Interiors</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>novaairllc.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>https://novaairllc.com/heat-pump-replacement-in-richardson-tx/</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Pump Replacement</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>salvasalce@novaairac.com</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>(214) 552-2008</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Richardson TX</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>100</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>heat pump installation Richardson TX</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 03:52 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L45"/>
+  <dimension ref="A1:L46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3078,6 +3078,66 @@
         </is>
       </c>
     </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Shadowcrest Roofing Inc</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>shadowcrestroofing.com</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>https://www.shadowcrestroofing.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Seam Copper</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>sales@shadowcrestroofing.com</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>(760) 593-0300</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>San Diego CA</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>90</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>metal roofing contractor San Diego CA</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 03:57 UTC (cycle 150)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:L47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3138,6 +3138,66 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>First Point Roofing</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>firstpointroof.com</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>https://www.firstpointroof.com/ocala</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>First Point</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>info@firstpointroof.com</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>(352) 729-1408</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>90</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>roofer Ocala FL</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 04:00 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L47"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3198,6 +3198,62 @@
         </is>
       </c>
     </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Home 1</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>plumbingsvc.com</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>https://plumbingsvc.com/</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>service@plumbingsvc.com</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>858.536.4161</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Sacramento CA</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>84</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>plumbing company Sacramento CA</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 04:10 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L48"/>
+  <dimension ref="A1:L49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3219,7 +3219,6 @@
           <t>https://plumbingsvc.com/</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>service@plumbingsvc.com</t>
@@ -3249,6 +3248,66 @@
         </is>
       </c>
       <c r="L48" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>San Antonio Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>san-antonio-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>http://www.san-antonio-metal-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Wind Damage</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>info@san-antonio-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>(726) 268-9896</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>88</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>metal roofing contractor San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 04:23 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L49"/>
+  <dimension ref="A1:L50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3313,6 +3313,66 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>American Energy Home Pros</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>americanenergyair.com</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>https://americanenergyair.com/ac-installation-elk-grove-ca/</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Trusted Sacramento</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>general@americanenergyair.com</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>(916) 520-9990</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>100</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>AC installation Elk Grove CA</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 04:35 UTC (cycle 176)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L50"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3373,6 +3373,62 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Your Favorite Roofer &amp; GC - Roofing in McKinney, TX</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>yfroofer.com</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>https://yfroofer.com/</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>admin@20if.clickwise.dev</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>(888) 596-7374</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>McKinney TX</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>88</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>roofer McKinney TX</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 04:44 UTC (cycle 182)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:L53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3394,7 +3394,6 @@
           <t>https://yfroofer.com/</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>admin@20if.clickwise.dev</t>
@@ -3424,6 +3423,126 @@
         </is>
       </c>
       <c r="L51" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Asheville Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>asheville-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>https://asheville-metal-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Metal Roofing</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>info@asheville-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>(828) 519-6016</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>100</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Asheville NC</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Jays Roofing</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>jaysroofingwnc.com</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>https://jaysroofingwnc.com/metal-roofing-contractor-asheville-nc/</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Owner Ac</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>jeff.jaysroofingwnc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>(828) 669-5629</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>100</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Asheville NC</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 04:49 UTC (cycle 186)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3548,6 +3548,66 @@
         </is>
       </c>
     </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>A/C Doctors</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>acdoctorsinc.com</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>https://acdoctorsinc.com/</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Doctors Inc</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>acdoctorsinc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>(772) 344-3944</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>100</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>HVAC contractor Port St Lucie FL</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 04:54 UTC (cycle 189)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L54"/>
+  <dimension ref="A1:L55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3608,6 +3608,66 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>American Rooter &amp; Drain</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>americanrooterdrain.com</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>https://americanrooterdrain.com/drain-cleaning/nampa/</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>American Rooter</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>ard@idahosplumber.com</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>(208) 366-5771</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Nampa ID</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>90</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>drain cleaning service Nampa ID</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 04:57 UTC (cycle 191)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3668,6 +3668,126 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Quality Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>qualityheat.net</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>https://www.qualityheat.net/fishers-in-heating-air-conditioning-contractor/</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Randy Swindle</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>qualityheat.cooling@gmail.com</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>317-791-4328</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Fishers IN</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>100</v>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>HVAC contractor Fishers IN</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Direct AC</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>directac.com</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>https://directac.com/hvac-services/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Serving Homeowners</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>info@directac.com</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>(800) 422-3325</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>94</v>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>heat pump installation Riverside CA</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 05:14 UTC (cycle 203)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3788,6 +3788,66 @@
         </is>
       </c>
     </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Alpine Roofing Specialists</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>alpineroofingspecialistsinc.com</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>https://alpineroofingspecialistsinc.com/service-areas/orem</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Roofing Specialists</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>alpineroofing@comcast.net</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>(801) 361-2301</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Orem UT</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
+        <v>90</v>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>roofing contractor Orem UT</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 05:16 UTC (cycle 204)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L58"/>
+  <dimension ref="A1:L59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3848,6 +3848,62 @@
         </is>
       </c>
     </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Air We Go</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>airwegoac.com</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>https://airwegoac.com/services/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>service@airwegoac.com</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>(561) 778-7078</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>90</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>heat pump installation West Palm Beach FL</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 10:41 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3869,7 +3869,6 @@
           <t>https://airwegoac.com/services/heat-pumps/</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>service@airwegoac.com</t>
@@ -3899,6 +3898,126 @@
         </is>
       </c>
       <c r="L59" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>O. S. Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>osheatingandcoolingservices.com</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>https://osheatingandcoolingservices.com/oakland-ca/</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Why Property</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>leslykvv@gmail.com</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>(510) 395-2895</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Oakland CA</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>100</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>heating and cooling company Oakland CA</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Throne Ranger Plumbing</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>thronerangerplumbing.com</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>https://www.thronerangerplumbing.com/southaven-ms</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Water Heater</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>contact@thronerangerplumbing.com</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>(901) 979-1727</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Southaven MS</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>80</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>plumbing company Southaven MS</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 10:42 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L61"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4023,6 +4023,118 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Texas Ace Heating and Air</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>texasacehvac.com</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>https://texasacehvac.com/ac-installation-in-arlington/</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>apply@texasacehvac.com</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>817.240.6701</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Arlington TX</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
+        <v>90</v>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>AC installation Arlington TX</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Air-Wave, New York's #1 Air Conditioning Specialist</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>airwaveac.com</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>https://www.airwaveac.com/</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>info@airwaveac.com</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>(718)-933-1011</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Bronx NY</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
+        <v>64</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>AC installation Bronx NY</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 10:45 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4044,7 +4044,6 @@
           <t>https://texasacehvac.com/ac-installation-in-arlington/</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>apply@texasacehvac.com</t>
@@ -4100,7 +4099,6 @@
           <t>https://www.airwaveac.com/</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>info@airwaveac.com</t>
@@ -4130,6 +4128,66 @@
         </is>
       </c>
       <c r="L63" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>CCY Roofing</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>ccyroofing.com</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>https://ccyroofing.com/augusta/</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Schedule My</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>office@ccyroofing.com</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>(706) 250-1859</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Augusta GA</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
+        <v>100</v>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>roof repair company Augusta GA</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 10:55 UTC (cycle 17)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L64"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4193,6 +4193,62 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Pacific Plumbing &amp; Drain Services</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>pacificplumbinganddrain.com</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>https://pacificplumbinganddrain.com/</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>info@pacificplumbinganddrain.com</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>(360) 684-1889</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Vancouver WA</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>100</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>plumber Vancouver WA</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 10:58 UTC (cycle 19)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L65"/>
+  <dimension ref="A1:L66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4214,7 +4214,6 @@
           <t>https://pacificplumbinganddrain.com/</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>info@pacificplumbinganddrain.com</t>
@@ -4244,6 +4243,62 @@
         </is>
       </c>
       <c r="L65" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Sanitary Sewer Service | FAYPWC.COM</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>faypwc.com</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>https://www.faypwc.com/sewer-service/</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>info@faypwc.com</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>(910) 483-1382</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>92</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>sewer repair Fayetteville NC</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 11:16 UTC (cycle 31)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:L67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4269,7 +4269,6 @@
           <t>https://www.faypwc.com/sewer-service/</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>info@faypwc.com</t>
@@ -4299,6 +4298,66 @@
         </is>
       </c>
       <c r="L66" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Ener-G Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>ener-ghvac.com</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>https://ener-ghvac.com/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Why Ocala</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>cool@ener-g-ac.com</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>(352) 843-7601</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>100</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>heating and cooling company Ocala FL</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 11:30 UTC (cycle 41)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L67"/>
+  <dimension ref="A1:L68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4363,6 +4363,66 @@
         </is>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Impact Roofing &amp; Renovation</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>impactrandr.com</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>https://impactrandr.com/round-rock/</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Impact Roofing</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>brandon@impactrandr.com</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>(512) 298-2086</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Round Rock TX</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>90</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>roofing contractor Round Rock TX</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 11:38 UTC (cycle 46)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L68"/>
+  <dimension ref="A1:L69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4423,6 +4423,66 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>aplusaircondition.com</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>aplusaircondition.com</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>https://aplusaircondition.com/ac-repair-Frisco-tx/</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Service Frisco</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>info@aplusaircondition.com</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>945-237-5986</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>90</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>air conditioning repair Frisco TX</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 11:45 UTC (cycle 51)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L69"/>
+  <dimension ref="A1:L70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4483,6 +4483,66 @@
         </is>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>All Seasons Heating, Cooling, and Plumbing | Hatfield MA</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>allseasonshvacp.com</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>https://allseasonshvacp.com/hvac-town/hvac-contractor-springfield-massachusetts/</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>All Seasons</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>office@allseasonshvacp.com</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>413.247.9842</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Springfield MA</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>90</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>HVAC contractor Springfield MA</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 11:49 UTC (cycle 54)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:L71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4543,6 +4543,66 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Plumber Las Vegas NV | Craig’s Plumbing</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>craigsplumbing.com</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>https://craigsplumbing.com/sewer-repair/</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Repair Process</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>hello@craigsplumbing.com</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>702-496-3892</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>90</v>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>sewer repair Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 11:57 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L71"/>
+  <dimension ref="A1:L73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4603,6 +4603,122 @@
         </is>
       </c>
     </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Rain City Pro -</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>raincitypro.com</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>https://raincitypro.com/air-conditioning-repair/</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>john@doe.com</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>(509) 236-4556</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Spokane WA</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>100</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>air conditioning repair Spokane WA</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Reputable Roofing &amp; Siding</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>reputableroofing.net</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>https://reputableroofing.net/aurora-il/</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Reputable Roof</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>ethan@reputableroofing.net</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>630-849-4548</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Aurora IL</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>90</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>residential roofing company Aurora IL</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 11:58 UTC (cycle 60)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L73"/>
+  <dimension ref="A1:L74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4624,7 +4624,6 @@
           <t>https://raincitypro.com/air-conditioning-repair/</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr">
         <is>
           <t>john@doe.com</t>
@@ -4714,6 +4713,62 @@
         </is>
       </c>
       <c r="L73" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>HVAC Contractor Oakland, CA | Anchor Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>anchorhvac.com</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>https://www.anchorhvac.com/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>info@anchorhvac.com</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>555-555-5555</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Oakland CA</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>88</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>HVAC contractor Oakland CA</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:03 UTC (cycle 63)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L74"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4739,7 +4739,6 @@
           <t>https://www.anchorhvac.com/</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr">
         <is>
           <t>info@anchorhvac.com</t>
@@ -4769,6 +4768,126 @@
         </is>
       </c>
       <c r="L74" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Delco Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>calldelco.com</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>https://calldelco.com/heatpumps-woodbridge-nj/</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Areas Products</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>johndoe@gmail.com</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>(732) 858-0453</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>100</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>heating and cooling company Woodbridge NJ</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Big League Roofers of Louisville</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>bigleaguerooferslouisville.com</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>https://bigleaguerooferslouisville.com/</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Service We</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>info@bigleaguerooferslouisville.com</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>(502) 876-7663</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Louisville KY</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>100</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>roofer Louisville KY</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:13 UTC (cycle 70)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4893,6 +4893,66 @@
         </is>
       </c>
     </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>S&amp;S HVAC</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>sandshvac.net</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>https://sandshvac.net/</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Lake Charles</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>operations@sandshvac.net</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>337-287-2132</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Lake Charles LA</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>100</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>heating and cooling company Lake Charles LA</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:16 UTC (cycle 72)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -4953,6 +4953,186 @@
         </is>
       </c>
     </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Marietta Plumber | Emergency Plumbing Services 24/7 | Paramount Plumbing</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ppatlanta.com</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>https://ppatlanta.com/plumber-marietta-ga</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Load More</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>paramount@paraplumbing.com</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>(404) 400-4444</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Marietta GA</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>100</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>emergency plumber Marietta GA</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Roof Repair Lee's Summit</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>leessummitroofrepair.com</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>https://leessummitroofrepair.com/</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Roof Repair</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>roofrepairleessummit@gmail.com</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>816-370-4326</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
+        <v>96</v>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>roof repair company Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Plumbers 4 Real</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>plumbers4real.com</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>https://plumbers4real.com/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Plumbing Answers</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>info@plumbers4real.com</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>(404) 819-2137</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>Marietta GA</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>90</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>emergency plumber Marietta GA</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:23 UTC (cycle 77)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5133,6 +5133,66 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Emergency Water Heater &amp; Sump Pump Repair – Naperville, IL</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>naperville-emergencyplumbing.com</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>https://naperville-emergencyplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Why Naperville</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>contact@naperville-emergencyplumbing.com</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>(630) 394-4247</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>Naperville IL</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>100</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>emergency plumber Naperville IL</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:36 UTC (cycle 86)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5193,6 +5193,66 @@
         </is>
       </c>
     </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Roof Repair Gulfport MS | Hurricane &amp; Leak Experts</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>roofrepairsquad.com</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>https://roofrepairsquad.com/roof-repair-gulfport-ms</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Orlando Sarasota</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>support@roofsquad.com</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>(866) 350-8889</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Gulfport MS</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>90</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>roof repair company Gulfport MS</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:39 UTC (cycle 88)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L82"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5253,6 +5253,126 @@
         </is>
       </c>
     </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Discount Drain Cleaning LV</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>discountdraincleanlv.com</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>https://discountdraincleanlv.com/service-areas/henderson-nv/drain-cleaning/</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Google Review</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>schedule@discountdraincleanlv.com</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>702-272-8743</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>Henderson NV</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
+        <v>100</v>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>drain cleaning service Henderson NV</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Aurora CO Sewer Repair | Sewer Line &amp; Camera Inspection | Oh Drain It</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ohdrainit.com</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>https://ohdrainit.com/sewer-repair-aurora.html</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Sewer Advisory</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>everettplumbinganddrain@gmail.com</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>(303) 253-7246</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>90</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>sewer repair Aurora CO</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:44 UTC (cycle 91)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L84"/>
+  <dimension ref="A1:L86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5373,6 +5373,126 @@
         </is>
       </c>
     </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>mtroofingokc</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>mtroofingokc.com</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>https://mtroofingokc.com/roofing-contractor-edmond-ok/</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Core Features</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>mtroofingokc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>(405) 832-0080</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
+        <v>100</v>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>roofing contractor Edmond OK</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Wright Way Roofing &amp; Construction -</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>wrightwayroofing.com</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>https://wrightwayroofing.com/roofing-contractor-in-edmond-ok/</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Wright Way</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>sales@wrightwayroofing.com</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>(405) 402-5075</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Edmond OK</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
+        <v>100</v>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>roofing contractor Edmond OK</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:51 UTC (cycle 96)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L86"/>
+  <dimension ref="A1:L87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5493,6 +5493,66 @@
         </is>
       </c>
     </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Plumbing Company | Philadelphia, PA | Greenjack Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>greenjackplumbing.com</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>https://www.greenjackplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Call Now</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>greenjackplumbingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>267-368-8373</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Philadelphia PA</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
+        <v>90</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>plumbing company Philadelphia PA</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:54 UTC (cycle 98)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5553,6 +5553,66 @@
         </is>
       </c>
     </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Greensboro Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>greensborometalroofing.com</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>https://www.greensborometalroofing.com/</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>At Greensboro</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>info@greensborometalroofing.com</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>(336) 203-1725</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Greensboro NC</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
+        <v>90</v>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Greensboro NC</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 12:57 UTC (cycle 100)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L88"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5613,6 +5613,66 @@
         </is>
       </c>
     </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>HVAC Company New Jersey</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>heat-pump-installation-toms-river.aeshvacnj.com</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>https://heat-pump-installation-toms-river.aeshvacnj.com/</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Call Us</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>example@mail.com</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>(888) 978-1291</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Toms River NJ</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
+        <v>100</v>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>heat pump installation Toms River NJ</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 13:00 UTC (cycle 102)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5673,6 +5673,66 @@
         </is>
       </c>
     </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Roof Repair Grand Rapids MI | Fast &amp; Reliable Residential Roof Repairs</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>completeroofingrepair.com</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>https://www.completeroofingrepair.com/roof-repair-grand-rapids-mi</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Roof Repair</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>info@completeroofingrepair.com</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>(616) 207-3831</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
+        <v>100</v>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>roof repair company Grand Rapids MI</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 13:06 UTC (cycle 106)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L90"/>
+  <dimension ref="A1:L91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5733,6 +5733,66 @@
         </is>
       </c>
     </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>I Know A Guy HVAC</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>iknowaguyhvac.com</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>http://www.iknowaguyhvac.com/heat-pump/installation</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Experience Free</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>admin@iknowaguyhvac.com</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>(385) 455-4700</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
+        <v>78</v>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>heat pump installation Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 13:14 UTC (cycle 112)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L91"/>
+  <dimension ref="A1:L92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5793,6 +5793,62 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Plumbing Services | York, PA | Rehm Plumbing</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>rehmplumbingheatinghvac.com</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>https://www.rehmplumbingheatinghvac.com/</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>rehmplumbing@aol.com</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>(717) 654-2433</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>York PA</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>88</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>plumber York PA</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 13:25 UTC (cycle 119)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L92"/>
+  <dimension ref="A1:L93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5814,7 +5814,6 @@
           <t>https://www.rehmplumbingheatinghvac.com/</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
           <t>rehmplumbing@aol.com</t>
@@ -5844,6 +5843,62 @@
         </is>
       </c>
       <c r="L92" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Central Air Installation Bangor, ME</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>fordhvac.com</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>https://www.fordhvac.com/central-air-installation-bangor-me/</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>info@fordhvac.com</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>(833) 435-3815</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Bangor ME</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
+        <v>90</v>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>AC installation Bangor ME</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 13:28 UTC (cycle 121)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L93"/>
+  <dimension ref="A1:L94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5869,7 +5869,6 @@
           <t>https://www.fordhvac.com/central-air-installation-bangor-me/</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="inlineStr">
         <is>
           <t>info@fordhvac.com</t>
@@ -5899,6 +5898,66 @@
         </is>
       </c>
       <c r="L93" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Recon Roofing &amp; Construction</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>reconroof.com</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>https://reconroof.com/</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Checklist For</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>info@reconroof.com</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>(515) 375-5437</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Des Moines IA</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
+        <v>98</v>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>roofing contractor Des Moines IA</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 13:31 UTC (cycle 123)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L94"/>
+  <dimension ref="A1:L95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -5963,6 +5963,66 @@
         </is>
       </c>
     </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Wasden Plumbing</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>wasdenplumbing.com</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>https://wasdenplumbing.com/emergency-plumbing-dallas-tx/</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Why Dallas</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>info@wasdenplumbing.com</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>214-364-6664</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Dallas TX</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
+        <v>100</v>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>emergency plumber Dallas TX</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 13:47 UTC (cycle 134)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L95"/>
+  <dimension ref="A1:L96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6023,6 +6023,66 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Pioneer Roofing</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>pioneerroofingcompany.com</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>https://www.pioneerroofingcompany.com/service-area/coral-springs-fl/</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>South Florida</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>yurimanuel@hotmail.es</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>954-737-1522</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
+        <v>88</v>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>residential roofing company Coral Springs FL</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 13:55 UTC (cycle 139)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L96"/>
+  <dimension ref="A1:L97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6083,6 +6083,62 @@
         </is>
       </c>
     </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Home - Metal Roofer Usa</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>metalrooferusa.com</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>https://www.metalrooferusa.com/</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>metalrooferusa@gmail.com</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>(818) 361-3631</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
+        <v>86</v>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Rancho Cucamonga CA</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:01 UTC (cycle 143)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L97"/>
+  <dimension ref="A1:L100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6104,7 +6104,6 @@
           <t>https://www.metalrooferusa.com/</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
           <t>metalrooferusa@gmail.com</t>
@@ -6134,6 +6133,182 @@
         </is>
       </c>
       <c r="L97" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Frisco No-Dig Pipe Repair</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>friscopiperepair.com</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>https://friscopiperepair.com/</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Request Free</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>dispatch@friscanodigpipe.com</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>(877) 552-8556</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Frisco TX</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>94</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>sewer repair Frisco TX</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ECS Roofing and Siding - Waukegan IL</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>ecsroofing.com</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>https://ecsroofing.com/</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>josh@ecsroofing.com</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>847-970-4500</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Waukegan IL</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>94</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>roofing contractor Waukegan IL</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Stanley Roofing Chicago</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>stanleyroofingchicago.com</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>https://stanleyroofingchicago.com/waukegan-il/</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Stanley Roofing</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>info@stanleyroofingchicago.com</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>896 105.0091</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Waukegan IL</t>
+        </is>
+      </c>
+      <c r="I100" t="n">
+        <v>90</v>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>roofing contractor Waukegan IL</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:03 UTC (cycle 145)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L100"/>
+  <dimension ref="A1:L102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6219,7 +6219,6 @@
           <t>https://ecsroofing.com/</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
       <c r="F99" t="inlineStr">
         <is>
           <t>josh@ecsroofing.com</t>
@@ -6309,6 +6308,122 @@
         </is>
       </c>
       <c r="L100" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Heat Pump Installation | Houston, TX</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>marcosac.com</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>https://www.marcosac.com/heat-pump-installation</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>office@marcosac.com</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>(346) 266-1769</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Houston TX</t>
+        </is>
+      </c>
+      <c r="I101" t="n">
+        <v>100</v>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>heat pump installation Houston TX</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>DPS Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>discountplumbingserviceinc.com</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>https://www.discountplumbingserviceinc.com/</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Discount Plumbing</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>discountplumbing20@gmail.com</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>435-673-3277</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>St George UT</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>90</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>plumbing company St George UT</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:06 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L102"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6334,7 +6334,6 @@
           <t>https://www.marcosac.com/heat-pump-installation</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
       <c r="F101" t="inlineStr">
         <is>
           <t>office@marcosac.com</t>
@@ -6424,6 +6423,62 @@
         </is>
       </c>
       <c r="L102" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Plumbing Services Tuscaloosa</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>jacobsplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>https://jacobsplumbinginc.com/areas-of-service/tuscaloosa-plumbing/</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>joannadjacobs@gmail.com</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>(205) 342-9994</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="I103" t="n">
+        <v>100</v>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>plumbing company Tuscaloosa AL</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:18 UTC (cycle 155)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L103"/>
+  <dimension ref="A1:L104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6449,7 +6449,6 @@
           <t>https://jacobsplumbinginc.com/areas-of-service/tuscaloosa-plumbing/</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
       <c r="F103" t="inlineStr">
         <is>
           <t>joannadjacobs@gmail.com</t>
@@ -6479,6 +6478,66 @@
         </is>
       </c>
       <c r="L103" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Metal Wholesale</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>metalwholesale.com</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>https://www.metalwholesale.com/manufacturer-location/cheyenne-wyoming</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Team Behind</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>sales@metalwholesalellc.com</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>(888)-509-4819</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="I104" t="n">
+        <v>84</v>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Cheyenne WY</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L104" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:20 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L104"/>
+  <dimension ref="A1:L106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6543,6 +6543,118 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Kalkbrenner Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>callkalkbrenner.com</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>https://callkalkbrenner.com/plumbing/water-heaters/</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>john@gmail.com</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>218-297-4342</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I105" t="n">
+        <v>94</v>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>water heater repair Duluth MN</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Lotta Hot Water</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>lottahotwater.com</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>https://lottahotwater.com/</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>lottahotwater@gmail.com</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>(218) 606-6177</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Duluth MN</t>
+        </is>
+      </c>
+      <c r="I106" t="n">
+        <v>80</v>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>water heater repair Duluth MN</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:21 UTC (cycle 157)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L106"/>
+  <dimension ref="A1:L107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6564,7 +6564,6 @@
           <t>https://callkalkbrenner.com/plumbing/water-heaters/</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
       <c r="F105" t="inlineStr">
         <is>
           <t>john@gmail.com</t>
@@ -6620,7 +6619,6 @@
           <t>https://lottahotwater.com/</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="inlineStr">
         <is>
           <t>lottahotwater@gmail.com</t>
@@ -6650,6 +6648,62 @@
         </is>
       </c>
       <c r="L106" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Sunset Air and Home Services</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>sunset-air.com</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>https://sunset-air.com/service-area/naples/</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>service@sunset-air.com</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>(239)-693-9005</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Naples FL</t>
+        </is>
+      </c>
+      <c r="I107" t="n">
+        <v>100</v>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>AC installation Naples FL</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L107" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:34 UTC (cycle 166)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L107"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6674,7 +6674,6 @@
           <t>https://sunset-air.com/service-area/naples/</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="inlineStr">
         <is>
           <t>service@sunset-air.com</t>
@@ -6704,6 +6703,66 @@
         </is>
       </c>
       <c r="L107" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Luxury Mechanical Systems</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>luxurymechanicalsystems.com</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>https://luxurymechanicalsystems.com/service-areas/sterling-heights/</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Services Most</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>service@luxurymechanicalsystems.com</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>(313) 512-6761</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="I108" t="n">
+        <v>90</v>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>furnace repair Sterling Heights MI</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:36 UTC (cycle 167)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L108"/>
+  <dimension ref="A1:L109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6768,6 +6768,66 @@
         </is>
       </c>
     </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Mitchell Heating</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>mitchellheating.com</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>https://mitchellheating.com/heat-pump-installation-aurora-co/</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Mitchell Heating</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>info@mitchellheating.com</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>719-596-6677</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>100</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>heat pump installation Aurora CO</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:37 UTC (cycle 168)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6828,6 +6828,122 @@
         </is>
       </c>
     </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Incredible Texas</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>incredibletexas.com</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>https://incredibletexas.com/best-roofing-contractors-in-corpus-christi-tx/</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Coastal Bend</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>incredibletexas@gmail.com</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>(361) 884-7663</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>100</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>residential roofing company Corpus Christi TX</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>G-Plumbing</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>gplumbingny.com</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>https://gplumbingny.com/</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>service.gplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>646-698-9036</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I111" t="n">
+        <v>90</v>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>emergency plumber Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:39 UTC (cycle 169)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L111"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6909,7 +6909,6 @@
           <t>https://gplumbingny.com/</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
         <is>
           <t>service.gplumbing@gmail.com</t>
@@ -6939,6 +6938,62 @@
         </is>
       </c>
       <c r="L111" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Auger's Plumbing</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>augersplumbinginc.com</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>https://augersplumbinginc.com/</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>sugersoffice@gmail.com</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>321-724-9174</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>90</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>plumbing company Palm Bay FL</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L112" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:40 UTC (cycle 170)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L112"/>
+  <dimension ref="A1:L113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -6964,7 +6964,6 @@
           <t>https://augersplumbinginc.com/</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr">
         <is>
           <t>sugersoffice@gmail.com</t>
@@ -6994,6 +6993,66 @@
         </is>
       </c>
       <c r="L112" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Stephens Roofing</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>stephensroofing.net</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>https://www.stephensroofing.net/</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>San Antonio</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>inquiries@stephensroofing.net</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>210-785-0994</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>San Antonio TX</t>
+        </is>
+      </c>
+      <c r="I113" t="n">
+        <v>100</v>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>roofer San Antonio TX</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L113" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:51 UTC (cycle 177)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L113"/>
+  <dimension ref="A1:L114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7058,6 +7058,66 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Bird's Eye Roofing Company</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>birdseyeroofing.com</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>https://birdseyeroofing.com/services/roof-replacement/</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Eye Roofing</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>info@birdseyeroofing.com</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>770.744.3358</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Roswell GA</t>
+        </is>
+      </c>
+      <c r="I114" t="n">
+        <v>100</v>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>roof replacement Roswell GA</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:55 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7118,6 +7118,58 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Stark Plumbing</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>starkplumbingllc.com</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>https://www.starkplumbingllc.com/</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>starkplumbingllc@gmail.com</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>Augusta GA</t>
+        </is>
+      </c>
+      <c r="I115" t="n">
+        <v>66</v>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>plumbing company Augusta GA</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 14:57 UTC (cycle 181)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L115"/>
+  <dimension ref="A1:L116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7139,13 +7139,11 @@
           <t>https://www.starkplumbingllc.com/</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="inlineStr">
         <is>
           <t>starkplumbingllc@gmail.com</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr"/>
       <c r="H115" t="inlineStr">
         <is>
           <t>Augusta GA</t>
@@ -7165,6 +7163,66 @@
         </is>
       </c>
       <c r="L115" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Metal Roofing Services Lees Summit, MO</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>roofingrpgs.com</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>https://lees-summit-mo.roofingrpgs.com/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>Lees Summit</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>info@roofingrpgs.com</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>(888) 766-0591</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="I116" t="n">
+        <v>90</v>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Lees Summit MO</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L116" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 15:01 UTC (cycle 183)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L116"/>
+  <dimension ref="A1:L117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7228,6 +7228,66 @@
         </is>
       </c>
     </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>VK Roofing</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>veirsklukroofing.com</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>https://veirsklukroofing.com/</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>Who We</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>info@vkrfg.com</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>(951) 781-9999</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>Riverside CA</t>
+        </is>
+      </c>
+      <c r="I117" t="n">
+        <v>76</v>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>roofer Riverside CA</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 15:04 UTC (cycle 185)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L117"/>
+  <dimension ref="A1:L118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7288,6 +7288,66 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>JL Brady</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>jlbradyco.com</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>https://www.jlbradyco.com/locations/davenport/furnace-repair-davenport/</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>Brady Company</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>jason@jlbradyco.com</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>309-865-5564</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>Davenport IA</t>
+        </is>
+      </c>
+      <c r="I118" t="n">
+        <v>100</v>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>furnace repair Davenport IA</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 15:08 UTC (cycle 188)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L118"/>
+  <dimension ref="A1:L119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7348,6 +7348,66 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Topper Construction</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>topperconstruction.com</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>https://www.topperconstruction.com/roofing/frederick-metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Tamko Master</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>info@topperconstruction.com</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>301-874-0220</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr">
+        <is>
+          <t>Frederick MD</t>
+        </is>
+      </c>
+      <c r="I119" t="n">
+        <v>90</v>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Frederick MD</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 15:18 UTC (cycle 195)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L119"/>
+  <dimension ref="A1:L120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7408,6 +7408,66 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Mr. Gates Heating and Cooling</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>mrgateshvac.com</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>https://www.mrgateshvac.com/air-conditioner-installation-las-vegas</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Las Vegas</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>mrgates702@gmail.com</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>(702) 600-3737</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr">
+        <is>
+          <t>Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="I120" t="n">
+        <v>90</v>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>AC installation Las Vegas NV</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 15:25 UTC (cycle 200)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L120"/>
+  <dimension ref="A1:L121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7468,6 +7468,66 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Moose Roofing</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>start.mooseroofing.com</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>https://www.start.mooseroofing.com/</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Educational Consultation</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>contactus@mooseroofing.com</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>402-763-4851</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr">
+        <is>
+          <t>Omaha NE</t>
+        </is>
+      </c>
+      <c r="I121" t="n">
+        <v>90</v>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>roof repair company Omaha NE</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 15:27 UTC (cycle 201)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L121"/>
+  <dimension ref="A1:L122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7528,6 +7528,66 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Residential &amp; Commercial Furnace Repair Lorain OH | Energy 1</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>energy1heating.com</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>https://www.energy1heating.com/furnace-repair</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>Fix My</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>alyczkowski@centurytel.net</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>(440) 986-5440</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr">
+        <is>
+          <t>Lorain OH</t>
+        </is>
+      </c>
+      <c r="I122" t="n">
+        <v>90</v>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>furnace repair Lorain OH</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 17:56 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L122"/>
+  <dimension ref="A1:L124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7588,6 +7588,126 @@
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Anything HVAC</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>anythinghvac.org</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>https://anythinghvac.org/</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>Operated Run</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>anythinghvacpa@gmail.com</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>(570) 335-3805</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr">
+        <is>
+          <t>Scranton PA</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>100</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>HVAC contractor Scranton PA</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Conroe Metal Roof Pros</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>metalroofingconroetx.com</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>https://metalroofingconroetx.com/</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Residential Metal</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>conroemetalroofpros@gmail.com</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>(936) 202-2476</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr">
+        <is>
+          <t>Conroe TX</t>
+        </is>
+      </c>
+      <c r="I124" t="n">
+        <v>90</v>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Conroe TX</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 17:57 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L124"/>
+  <dimension ref="A1:L125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7708,6 +7708,66 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Town &amp; Country Roofing and Restoration</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>town-countryroofing.com</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>https://town-countryroofing.com/fayetteville-ar/</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>For Fayetteville</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>townandcountryroofingar@gmail.com</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>(479) 310-9693</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr">
+        <is>
+          <t>Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="I125" t="n">
+        <v>100</v>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>roofing contractor Fayetteville AR</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:00 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L125"/>
+  <dimension ref="A1:L127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7768,6 +7768,122 @@
         </is>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Armor Roofing LLC</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>armorbuilder.com</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>https://armorbuilder.com/roof-replacement-durham-nc/</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Robert Lopez</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>ar@armorbuilder.com</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>336-999-4940</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>100</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>roof replacement Durham NC</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L126" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Recovery Roofing of NC, LLC</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>recoveryroofingnc.com</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>https://recoveryroofingnc.com/</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>mlodata@recoveryroofingnc.com</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>919-371-8990</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>90</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>roof replacement Durham NC</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:02 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L127"/>
+  <dimension ref="A1:L128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7849,7 +7849,6 @@
           <t>https://recoveryroofingnc.com/</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
       <c r="F127" t="inlineStr">
         <is>
           <t>mlodata@recoveryroofingnc.com</t>
@@ -7879,6 +7878,66 @@
         </is>
       </c>
       <c r="L127" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Nathan's Roof Repairs</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>nathansroofrepairs.com</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>https://nathansroofrepairs.com/</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Team Nathan</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>support@nathansroofrepairs.com</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>(804) 273-9200</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I128" t="n">
+        <v>100</v>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>roof repair company Richmond VA</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L128" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:03 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L128"/>
+  <dimension ref="A1:L130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -7943,6 +7943,122 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Guardian Roofing and Remodeling</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>guardianrtx.com</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>https://guardianrtx.com/all-locations/new-braunfels-roofing-and-home-remodeling-company/</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>New Braunfels</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>info.guardiantx@gmail.com</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>(210)-864-1937</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="I129" t="n">
+        <v>100</v>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>roof repair company New Braunfels TX</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L129" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Metal Roof Albuquerque</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>metalroofalbuquerque.com</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>http://www.metalroofalbuquerque.com/</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofalbuquerque.com</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>866-868-1006</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="I130" t="n">
+        <v>84</v>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Albuquerque NM</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:08 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L130"/>
+  <dimension ref="A1:L131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8024,7 +8024,6 @@
           <t>http://www.metalroofalbuquerque.com/</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
       <c r="F130" t="inlineStr">
         <is>
           <t>moreinfo@metalroofalbuquerque.com</t>
@@ -8054,6 +8053,62 @@
         </is>
       </c>
       <c r="L130" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Westminster, CO Plumbing and Drain Cleaning | Mile High Drain</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>milehighdrain.com</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>https://www.milehighdrain.com/westminster</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>office@milehighdrain.com</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>303-726-3888</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Westminster CO</t>
+        </is>
+      </c>
+      <c r="I131" t="n">
+        <v>90</v>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>drain cleaning service Westminster CO</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:18 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L131"/>
+  <dimension ref="A1:L132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8079,7 +8079,6 @@
           <t>https://www.milehighdrain.com/westminster</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
       <c r="F131" t="inlineStr">
         <is>
           <t>office@milehighdrain.com</t>
@@ -8109,6 +8108,66 @@
         </is>
       </c>
       <c r="L131" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Roof Repair Durham</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>roofrepair-durham.com</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>https://roofrepair-durham.com/</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Roofing Service</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>arhamsarfraz80@gmail.com</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>984-230-5620</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Durham NC</t>
+        </is>
+      </c>
+      <c r="I132" t="n">
+        <v>90</v>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>roof repair company Durham NC</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:21 UTC (cycle 18)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L132"/>
+  <dimension ref="A1:L133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8173,6 +8173,66 @@
         </is>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Rocket Roofing</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>rocketroofingne.com</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>https://www.rocketroofingne.com/location/bellevue</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Storm Damage</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>contact@rocketroofingne.com</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>(402) 291-8888</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>Bellevue NE</t>
+        </is>
+      </c>
+      <c r="I133" t="n">
+        <v>90</v>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>roof repair company Bellevue NE</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:24 UTC (cycle 20)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L133"/>
+  <dimension ref="A1:L134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8233,6 +8233,66 @@
         </is>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>fort-lauderdale-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>https://fort-lauderdale-metal-roofing.com/</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>info@fort-lauderdale-metal-roofing.com</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>(754) 354-5057</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="I134" t="n">
+        <v>100</v>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Fort Lauderdale FL</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:36 UTC (cycle 28)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L134"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8293,6 +8293,66 @@
         </is>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Thermostat Masters</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>thermostatmasters.com</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>https://thermostatmasters.com/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Surrounding Areas</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>contact@thermostatmasters.com</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>(919)219.9810</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>Raleigh NC</t>
+        </is>
+      </c>
+      <c r="I135" t="n">
+        <v>100</v>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>AC installation Raleigh NC</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:51 UTC (cycle 38)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L135"/>
+  <dimension ref="A1:L136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8353,6 +8353,66 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Cook Bros Roofing</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>cookbrosroofing.com</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>https://cookbrosroofing.com/services/metal-roofing/florida/miramar</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Standard Dedicated</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>hello@cookbrosroofing.com</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>(877) 385-3819</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>Miramar FL</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>90</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Miramar FL</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:54 UTC (cycle 40)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L136"/>
+  <dimension ref="A1:L137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8413,6 +8413,66 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Roofing in Ankeny, IA — Platinum Roofing &amp; Contracting</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>platinumroofingiowa.com</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>https://www.platinumroofingiowa.com/roofing/ankeny/</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>West Des</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>info@prcia.com</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>(515) 975-8632</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Ankeny IA</t>
+        </is>
+      </c>
+      <c r="I137" t="n">
+        <v>80</v>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>roofer Ankeny IA</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 18:58 UTC (cycle 43)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L137"/>
+  <dimension ref="A1:L138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8473,6 +8473,66 @@
         </is>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Pickwick Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>pickwickpros.com</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>https://pickwickpros.com/local-plumber/plumber-norwalk-ct/</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>East Norwalk</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>info@pickwickpros.com</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>(203)531-6100</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Norwalk CT</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>90</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>plumber Norwalk CT</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 19:00 UTC (cycle 44)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L138"/>
+  <dimension ref="A1:L139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8533,6 +8533,66 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Rainy Day Restoration and Roofing</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>rainydayrestoration.com</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>https://rainydayrestoration.com/roof-repair-in-plano-tx/</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Rainy Day</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>info@rainydayservices.com</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>(972) 747-7734</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>Plano TX</t>
+        </is>
+      </c>
+      <c r="I139" t="n">
+        <v>90</v>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>roof repair company Plano TX</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 19:01 UTC (cycle 45)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L139"/>
+  <dimension ref="A1:L140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8593,6 +8593,66 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Temperstead Heating &amp; Air</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>temperstead.com</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>https://temperstead.com/services/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Twin Cities</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>justin@temperstead.com</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>(612) 688-5332</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>St Paul MN</t>
+        </is>
+      </c>
+      <c r="I140" t="n">
+        <v>90</v>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>AC installation St Paul MN</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 19:22 UTC (cycle 59)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L140"/>
+  <dimension ref="A1:L141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8653,6 +8653,62 @@
         </is>
       </c>
     </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Atlanta Heat Pump Installation and Heat Pump Installation Near Me |Atlanta HVAC </t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>atlantahvacpros.com</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>https://atlantahvacpros.com/services/heat-pump-install.html</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>contact@atlantahvacpros.com</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>(404)-962-0203</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Atlanta GA</t>
+        </is>
+      </c>
+      <c r="I141" t="n">
+        <v>90</v>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>heat pump installation Atlanta GA</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 19:29 UTC (cycle 64)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L141"/>
+  <dimension ref="A1:L144"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8674,7 +8674,6 @@
           <t>https://atlantahvacpros.com/services/heat-pump-install.html</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
       <c r="F141" t="inlineStr">
         <is>
           <t>contact@atlantahvacpros.com</t>
@@ -8704,6 +8703,182 @@
         </is>
       </c>
       <c r="L141" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>One Source Roofing &amp; Maintenance LLC</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>onesourceroofinglansing.com</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>https://onesourceroofinglansing.com/commercial-roofing-services/metal-roofing/</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr"/>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>info@onesourceroofinglansing.com</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>(517) 231-9196</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I142" t="n">
+        <v>100</v>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Lansing MI</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Anchor Siding LLC</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>anchorconstructionmi.com</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>https://anchorconstructionmi.com/service-areas/ingham-county/lansing/metal-roofing-in-lansing/</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Andrew Byrum</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>info@anchorconstructionmi.com</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>(989) 900-0018</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>90</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Lansing MI</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>One &amp; Done Metal Roofing</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>oneanddonemetalroofing.com</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>https://oneanddonemetalroofing.com/</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Answers Do</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>sales@oneanddonemetalroofing.com</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>(517) 291-8049</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I144" t="n">
+        <v>84</v>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Lansing MI</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 19:40 UTC (cycle 71)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L144"/>
+  <dimension ref="A1:L145"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8729,7 +8729,6 @@
           <t>https://onesourceroofinglansing.com/commercial-roofing-services/metal-roofing/</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>info@onesourceroofinglansing.com</t>
@@ -8879,6 +8878,62 @@
         </is>
       </c>
       <c r="L144" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Arizona EZ AC</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>azezac.com</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>https://azezac.com/</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>info@azezac.com</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>(480) 660-6604</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Chandler AZ</t>
+        </is>
+      </c>
+      <c r="I145" t="n">
+        <v>100</v>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>AC installation Chandler AZ</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 19:46 UTC (cycle 75)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L145"/>
+  <dimension ref="A1:L146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8904,7 +8904,6 @@
           <t>https://azezac.com/</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
       <c r="F145" t="inlineStr">
         <is>
           <t>info@azezac.com</t>
@@ -8934,6 +8933,62 @@
         </is>
       </c>
       <c r="L145" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Emmanuel's Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>emmanuelshac.com</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>https://www.emmanuelshac.com/</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>emmanuelshac@gmail.com</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>(224) 513-1181</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Waukegan IL</t>
+        </is>
+      </c>
+      <c r="I146" t="n">
+        <v>100</v>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>AC installation Waukegan IL</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 19:47 UTC (cycle 76)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L146"/>
+  <dimension ref="A1:L147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -8959,7 +8959,6 @@
           <t>https://www.emmanuelshac.com/</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
       <c r="F146" t="inlineStr">
         <is>
           <t>emmanuelshac@gmail.com</t>
@@ -8989,6 +8988,66 @@
         </is>
       </c>
       <c r="L146" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Summit Roofing</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>summitroofingslc.com</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>https://summitroofingslc.com/</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>City Byron</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>byron@summitroofingslc.com</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>(385) 601-2262</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="I147" t="n">
+        <v>100</v>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>roofing contractor Salt Lake City UT</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 19:54 UTC (cycle 81)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L147"/>
+  <dimension ref="A1:L150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9053,6 +9053,182 @@
         </is>
       </c>
     </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Scottsdale AC Pros</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>scottsdaleacpros.com</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>https://scottsdaleacpros.com/services/ac-installation/</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Lead Technician</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>admin@scottsdaleacpros.com</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>(602) 960-7890</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>Scottsdale AZ</t>
+        </is>
+      </c>
+      <c r="I148" t="n">
+        <v>90</v>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>AC installation Scottsdale AZ</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>SoCal Emergency Plumbing Mission Viejo</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>socalemergencyplumbingmissionviejo.com</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>https://socalemergencyplumbingmissionviejo.com/service-areas/fontana</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Mission Viejo</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>info@socalemergencyplumbingmissionviejo.com</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>(949) 951-1277</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Fontana CA</t>
+        </is>
+      </c>
+      <c r="I149" t="n">
+        <v>90</v>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>emergency plumber Fontana CA</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Air Conditioner Installation and Replacement in Lansing, MI | Top-rated AC repai</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>butlerheatingairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>https://butlerheatingairconditioning.com/lansing-air-conditioner-installation-and-replacement</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>office@butlerheatingairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>(517) 256-9524</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>Lansing MI</t>
+        </is>
+      </c>
+      <c r="I150" t="n">
+        <v>90</v>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>AC installation Lansing MI</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 20:09 UTC (cycle 91)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L150"/>
+  <dimension ref="A1:L151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9194,7 +9194,6 @@
           <t>https://butlerheatingairconditioning.com/lansing-air-conditioner-installation-and-replacement</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
       <c r="F150" t="inlineStr">
         <is>
           <t>office@butlerheatingairconditioning.com</t>
@@ -9224,6 +9223,66 @@
         </is>
       </c>
       <c r="L150" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Top-Rated HVAC Services in Brockton, MA</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>jarvishvac.com</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>https://jarvishvac.com/brockton-ma.html</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Locally Owned</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>jarvishvacr@gmail.com</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>(774) 339-5252</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Brockton MA</t>
+        </is>
+      </c>
+      <c r="I151" t="n">
+        <v>100</v>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>air conditioning repair Brockton MA</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 20:11 UTC (cycle 92)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L151"/>
+  <dimension ref="A1:L152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9288,6 +9288,66 @@
         </is>
       </c>
     </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>ocalalinerepair.com</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>https://ocalalinerepair.com/</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Licensed We</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>help@ocala.pro</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>352-555-0199</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>Ocala FL</t>
+        </is>
+      </c>
+      <c r="I152" t="n">
+        <v>62</v>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>sewer repair Ocala FL</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 20:15 UTC (cycle 95)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L152"/>
+  <dimension ref="A1:L153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9348,6 +9348,66 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>B&amp;D HVAC</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>banddheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>https://banddheatingandcooling.com/</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Highly Recommended</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>bdheating23@gmail.com</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>(615) 834-4006</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>Nashville TN</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>100</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>heating and cooling company Nashville TN</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 20:21 UTC (cycle 99)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L153"/>
+  <dimension ref="A1:L154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9408,6 +9408,66 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Commercial Metal Roofer | Sandy Springs, GA | McNail Brothers</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>mcnailbrothers.com</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>https://www.mcnailbrothers.com/sap/commercial-metal-roofer/sandy-springs-ga</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Watch Video</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>info@mcnailbrothers.com</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>(770) 828-7614</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="I154" t="n">
+        <v>98</v>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Sandy Springs GA</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 20:30 UTC (cycle 105)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L154"/>
+  <dimension ref="A1:L156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9468,6 +9468,126 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Cool Roofs</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>coolroofs.co</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>https://coolroofs.co/location/beaumont/</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Home About</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>info@coolroofs.co</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>409-710-5041</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>Beaumont TX</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>90</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>residential roofing company Beaumont TX</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Desert Rain Plumbing</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>desertrainplumbing.com</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>https://desertrainplumbing.com/emergency-plumber-surprise.html</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Desert Rain</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>office@desertrainplumbing.com</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>(480) 675-7861</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>Surprise AZ</t>
+        </is>
+      </c>
+      <c r="I156" t="n">
+        <v>90</v>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>emergency plumber Surprise AZ</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 20:33 UTC (cycle 107)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L156"/>
+  <dimension ref="A1:L157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9588,6 +9588,66 @@
         </is>
       </c>
     </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Bell Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>bellheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>https://bellheatingandcooling.com/hvac-wichita-ks/</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Keep Your</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>bell.hvac2022@gmail.com</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>(620) 899-5574</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I157" t="n">
+        <v>100</v>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>AC installation Wichita KS</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 20:40 UTC (cycle 112)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L157"/>
+  <dimension ref="A1:L158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9648,6 +9648,66 @@
         </is>
       </c>
     </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>HVAC Billings MT | Heating &amp; Cooling Service</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>laurelhvac.com</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>https://laurelhvac.com/billings-mt</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>Yellowstone County</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>info@laurelhvac.com</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>(406) 876-5585</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>Billings MT</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>86</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>heating and cooling company Billings MT</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:00 UTC (cycle 125)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L158"/>
+  <dimension ref="A1:L160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9708,6 +9708,118 @@
         </is>
       </c>
     </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t xml:space="preserve">J &amp; L Heating &amp; Air Conditioning - Top Rated HVAC Contractor - Pawtucket, Rhode </t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>jandlheatingandac.com</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>https://www.jandlheatingandac.com/</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>lmss1968@hotmail.com</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>401-617-1275</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>Pawtucket RI</t>
+        </is>
+      </c>
+      <c r="I159" t="n">
+        <v>100</v>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>heating and cooling company Pawtucket RI</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Residential Roofing company Torrance (424) 800-9880</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>torranceroofing.us</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>https://www.torranceroofing.us/residential-roofing-torrance-ca</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>info@torranceroofing.us</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>(424) 800-9880</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>98</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>residential roofing company Torrance CA</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:03 UTC (cycle 127)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L160"/>
+  <dimension ref="A1:L161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9729,7 +9729,6 @@
           <t>https://www.jandlheatingandac.com/</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
       <c r="F159" t="inlineStr">
         <is>
           <t>lmss1968@hotmail.com</t>
@@ -9785,7 +9784,6 @@
           <t>https://www.torranceroofing.us/residential-roofing-torrance-ca</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
       <c r="F160" t="inlineStr">
         <is>
           <t>info@torranceroofing.us</t>
@@ -9815,6 +9813,66 @@
         </is>
       </c>
       <c r="L160" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>ABCO Air</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>abcoair.com</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://www.abcoair.com/</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>Fred Robanser</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>abco@abcoair.com</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>415-648-7135</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>San Francisco CA</t>
+        </is>
+      </c>
+      <c r="I161" t="n">
+        <v>78</v>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>HVAC contractor San Francisco CA</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:16 UTC (cycle 136)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L161"/>
+  <dimension ref="A1:L162"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9878,6 +9878,66 @@
         </is>
       </c>
     </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Roofing &amp; Sheet Metal Services | St. Paul &amp; Minneapolis</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>berwaldroofing.com</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>https://www.berwaldroofing.com/</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>Residential Metal</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>info@berwaldsroofing.com</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>651-777-7411</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>St Paul MN</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>100</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>metal roofing contractor St Paul MN</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:32 UTC (cycle 147)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L162"/>
+  <dimension ref="A1:L163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9938,6 +9938,62 @@
         </is>
       </c>
     </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Frontera Refrigeration, LLC</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>fronterarefrigeration.com</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>https://fronterarefrigeration.com/heating/furnace-repair/</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>info@fronterarefrigeration.com</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>(915) 238-0970</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>El Paso TX</t>
+        </is>
+      </c>
+      <c r="I163" t="n">
+        <v>90</v>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>furnace repair El Paso TX</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:33 UTC (cycle 148)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L163"/>
+  <dimension ref="A1:L164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -9959,7 +9959,6 @@
           <t>https://fronterarefrigeration.com/heating/furnace-repair/</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
       <c r="F163" t="inlineStr">
         <is>
           <t>info@fronterarefrigeration.com</t>
@@ -9989,6 +9988,58 @@
         </is>
       </c>
       <c r="L163" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>AC Installation Austin | AC Install &amp; Replacement Austin, TX</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>acinstallationaustin.com</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>https://acinstallationaustin.com/</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>info@acinstallationaustin.com</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr"/>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>Austin TX</t>
+        </is>
+      </c>
+      <c r="I164" t="n">
+        <v>76</v>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>AC installation Austin TX</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:38 UTC (cycle 151)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L164"/>
+  <dimension ref="A1:L165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10014,13 +10014,11 @@
           <t>https://acinstallationaustin.com/</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
       <c r="F164" t="inlineStr">
         <is>
           <t>info@acinstallationaustin.com</t>
         </is>
       </c>
-      <c r="G164" t="inlineStr"/>
       <c r="H164" t="inlineStr">
         <is>
           <t>Austin TX</t>
@@ -10040,6 +10038,66 @@
         </is>
       </c>
       <c r="L164" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>metalroofingspokanewa.net</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>metalroofingspokanewa.net</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>https://metalroofingspokanewa.net/</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>Projects Completed</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>roofed@metalroofingspokanewa.com</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>509-355-3998</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>Spokane WA</t>
+        </is>
+      </c>
+      <c r="I165" t="n">
+        <v>88</v>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Spokane WA</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:39 UTC (cycle 152)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L165"/>
+  <dimension ref="A1:L166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10103,6 +10103,62 @@
         </is>
       </c>
     </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Honest Co HVAC, LLC</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>honestcohvacllc.com</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>https://www.honestcohvacllc.com/</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>hunter@honestcohvac.com</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>(316) 648-7311</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>Wichita KS</t>
+        </is>
+      </c>
+      <c r="I166" t="n">
+        <v>100</v>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>HVAC contractor Wichita KS</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:41 UTC (cycle 153)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L166"/>
+  <dimension ref="A1:L168"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10124,7 +10124,6 @@
           <t>https://www.honestcohvacllc.com/</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
       <c r="F166" t="inlineStr">
         <is>
           <t>hunter@honestcohvac.com</t>
@@ -10154,6 +10153,126 @@
         </is>
       </c>
       <c r="L166" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Minnesota Site</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>mnroofingco.com</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>https://www.mnroofingco.com/</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>Roofing Company</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>info@mnroofingco.com</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>(612) 888-7663</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I167" t="n">
+        <v>100</v>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>roof replacement Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Roof Replacement Minneapolis  |  Advanced Exteriors MN Roofer</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>advancedexteriorsmn.com</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>https://www.advancedexteriorsmn.com/</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Minneapolis Cost</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>cmarkus@advancedexteriorsmn.com</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>(763) 537-5117</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="I168" t="n">
+        <v>90</v>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>roof replacement Minneapolis MN</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:42 UTC (cycle 154)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L168"/>
+  <dimension ref="A1:L169"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10278,6 +10278,66 @@
         </is>
       </c>
     </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Reasonable Air LLC — HVAC Services in Summerville &amp; the SC Lowcountry</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>reasonableairofsc.com</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>https://www.reasonableairofsc.com/</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>Reasonable Air</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>contactus@reasonableairofsc.com</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>(843) 900-4799</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>Summerville SC</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>90</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>AC installation Summerville SC</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:45 UTC (cycle 156)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L169"/>
+  <dimension ref="A1:L170"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10338,6 +10338,66 @@
         </is>
       </c>
     </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>1213 Plumbing LLC</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>1213plumbing.com</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>https://www.1213plumbing.com/services/plumber/emergency-plumbing-24-7</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Client Reviews</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>rudy.bustamante@yahoo.com</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>(806) 782-7454</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>Lubbock TX</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>100</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>emergency plumber Lubbock TX</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 21:50 UTC (cycle 159)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L170"/>
+  <dimension ref="A1:L173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10398,6 +10398,186 @@
         </is>
       </c>
     </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Metal Roof Installation Services | Greenville County, SC</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>callontop.com</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>https://www.callontop.com/metal-roof-installation</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>Lifetime Metal</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>bill@callontop.com</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>(864) 887-3509</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>100</v>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Greenville SC</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Affordable Roofing</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>affordableroofingsc.com</t>
+        </is>
+      </c>
+      <c r="D172" t="inlineStr">
+        <is>
+          <t>https://affordableroofingsc.com/services/metal-roof/</t>
+        </is>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>Roof Flashing</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>info@youraffordableroof.com</t>
+        </is>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>(864)859-9002</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>90</v>
+      </c>
+      <c r="J172" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Greenville SC</t>
+        </is>
+      </c>
+      <c r="K172" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Piper Roofing</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>piperroofing.com</t>
+        </is>
+      </c>
+      <c r="D173" t="inlineStr">
+        <is>
+          <t>https://www.piperroofing.com/roof-services/metal-roofs</t>
+        </is>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>Piper Award</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>info@piperroofing.com</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>864-269-6645</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>Greenville SC</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>86</v>
+      </c>
+      <c r="J173" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Greenville SC</t>
+        </is>
+      </c>
+      <c r="K173" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 22:02 UTC (cycle 167)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L173"/>
+  <dimension ref="A1:L174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10578,6 +10578,62 @@
         </is>
       </c>
     </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Babov LLC</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>babov-llc.com</t>
+        </is>
+      </c>
+      <c r="D174" t="inlineStr">
+        <is>
+          <t>https://babov-llc.com/service-area/worcester-ma/roofing/</t>
+        </is>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>Service Area</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>info@babov-llc.com</t>
+        </is>
+      </c>
+      <c r="G174" t="inlineStr"/>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>Worcester MA</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>86</v>
+      </c>
+      <c r="J174" t="inlineStr">
+        <is>
+          <t>roof replacement Worcester MA</t>
+        </is>
+      </c>
+      <c r="K174" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 22:21 UTC (cycle 180)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L174"/>
+  <dimension ref="A1:L175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10609,7 +10609,6 @@
           <t>info@babov-llc.com</t>
         </is>
       </c>
-      <c r="G174" t="inlineStr"/>
       <c r="H174" t="inlineStr">
         <is>
           <t>Worcester MA</t>
@@ -10629,6 +10628,62 @@
         </is>
       </c>
       <c r="L174" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Hillsboro Heating Ventilation and Air Conditioning</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>hillsboroheating.com</t>
+        </is>
+      </c>
+      <c r="D175" t="inlineStr">
+        <is>
+          <t>https://www.hillsboroheating.com/company/</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>info@hillsboro.com</t>
+        </is>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>(503)746-7229</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>90</v>
+      </c>
+      <c r="J175" t="inlineStr">
+        <is>
+          <t>heating and cooling company Hillsboro OR</t>
+        </is>
+      </c>
+      <c r="K175" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L175" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 22:47 UTC (cycle 198)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L175"/>
+  <dimension ref="A1:L176"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10654,7 +10654,6 @@
           <t>https://www.hillsboroheating.com/company/</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
       <c r="F175" t="inlineStr">
         <is>
           <t>info@hillsboro.com</t>
@@ -10684,6 +10683,66 @@
         </is>
       </c>
       <c r="L175" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Plumbfast Emergency Plumbing</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>plumbfastcolorado.com</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr">
+        <is>
+          <t>https://plumbfastcolorado.com/</t>
+        </is>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>Emergency Plumbing</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>plumbfastcolorado@gmail.com</t>
+        </is>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>983-955-2226</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>Aurora CO</t>
+        </is>
+      </c>
+      <c r="I176" t="n">
+        <v>90</v>
+      </c>
+      <c r="J176" t="inlineStr">
+        <is>
+          <t>emergency plumber Aurora CO</t>
+        </is>
+      </c>
+      <c r="K176" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L176" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 23:35 UTC (cycle 2)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L176"/>
+  <dimension ref="A1:L178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10748,6 +10748,122 @@
         </is>
       </c>
     </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Victor Sewer and Drain Services</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>victorsewer.com</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>https://www.victorsewer.com/</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>Understanding Tree</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>example@mysite.com</t>
+        </is>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>(718) 645-6711</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>100</v>
+      </c>
+      <c r="J177" t="inlineStr">
+        <is>
+          <t>drain cleaning service Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K177" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>NY Sewer and Drain</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>nysewerdrain.com</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>https://www.nysewerdrain.com/brooklyn</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>info@nysewerdrain.com</t>
+        </is>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>(718) 337-8330</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>90</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>drain cleaning service Brooklyn NY</t>
+        </is>
+      </c>
+      <c r="K178" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 23:40 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L178"/>
+  <dimension ref="A1:L179"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10829,7 +10829,6 @@
           <t>https://www.nysewerdrain.com/brooklyn</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
       <c r="F178" t="inlineStr">
         <is>
           <t>info@nysewerdrain.com</t>
@@ -10859,6 +10858,62 @@
         </is>
       </c>
       <c r="L178" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Roofing | Sparks, NV | Gurrs Roofing Heating and Sheet Metal</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>gurrsroofing.com</t>
+        </is>
+      </c>
+      <c r="D179" t="inlineStr">
+        <is>
+          <t>https://www.gurrsroofing.com/</t>
+        </is>
+      </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>gurrsroofing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>775-358-1711</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>Sparks NV</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>88</v>
+      </c>
+      <c r="J179" t="inlineStr">
+        <is>
+          <t>roofer Sparks NV</t>
+        </is>
+      </c>
+      <c r="K179" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L179" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 23:41 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L179"/>
+  <dimension ref="A1:L180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10884,7 +10884,6 @@
           <t>https://www.gurrsroofing.com/</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
       <c r="F179" t="inlineStr">
         <is>
           <t>gurrsroofing@gmail.com</t>
@@ -10914,6 +10913,66 @@
         </is>
       </c>
       <c r="L179" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Greenfox Services</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>greenfoxservices.com</t>
+        </is>
+      </c>
+      <c r="D180" t="inlineStr">
+        <is>
+          <t>https://greenfoxservices.com/residential/heat-pumps/</t>
+        </is>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>Owner Mr</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr">
+        <is>
+          <t>info@greenfoxservices.com</t>
+        </is>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>410-992-8200</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>Columbia MD</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>90</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>heat pump installation Columbia MD</t>
+        </is>
+      </c>
+      <c r="K180" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L180" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-09-29 23:44 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L180"/>
+  <dimension ref="A1:L181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10978,6 +10978,62 @@
         </is>
       </c>
     </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Integrity Home Services</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>integrityheatandair.com</t>
+        </is>
+      </c>
+      <c r="D181" t="inlineStr">
+        <is>
+          <t>https://integrityheatandair.com/hvac-services/heat-pump-installation/</t>
+        </is>
+      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>info@integrityheatandair.com</t>
+        </is>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>(405) 913-7167</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>100</v>
+      </c>
+      <c r="J181" t="inlineStr">
+        <is>
+          <t>heat pump installation Oklahoma City OK</t>
+        </is>
+      </c>
+      <c r="K181" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-09-29 23:56 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-09-29.xlsx
+++ b/output/leads_2026-09-29.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L181"/>
+  <dimension ref="A1:L182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -10999,7 +10999,6 @@
           <t>https://integrityheatandair.com/hvac-services/heat-pump-installation/</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
       <c r="F181" t="inlineStr">
         <is>
           <t>info@integrityheatandair.com</t>
@@ -11029,6 +11028,66 @@
         </is>
       </c>
       <c r="L181" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>JL Cooling &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>jlcandh.com</t>
+        </is>
+      </c>
+      <c r="D182" t="inlineStr">
+        <is>
+          <t>https://jlcandh.com/ac-repair-mcallen-tx/</t>
+        </is>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>South Texas</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr">
+        <is>
+          <t>jovan@jlcandh.com</t>
+        </is>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>956-569-4838</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>McAllen TX</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>86</v>
+      </c>
+      <c r="J182" t="inlineStr">
+        <is>
+          <t>air conditioning repair McAllen TX</t>
+        </is>
+      </c>
+      <c r="K182" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L182" t="inlineStr">
         <is>
           <t>2026-09-29</t>
         </is>

</xml_diff>